<commit_message>
feat: added ENG ambience data
</commit_message>
<xml_diff>
--- a/exp/jack/Data/UK_Data/TABULA_to_UWE.xlsx
+++ b/exp/jack/Data/UK_Data/TABULA_to_UWE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/jjjl4_cam_ac_uk/Documents/1. Cambridge/1. PhD/1. Projects/10.EP/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JackLynch/CUBES/exp/jack/Data/UK_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C36F2BA-6B35-EC4B-A425-26472FB447FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7CC380-D0CA-F04B-9F5C-F3C972C64874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="14000" xr2:uid="{7F739DF3-AE70-5648-ABAC-6400F7C2E419}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="14000" activeTab="1" xr2:uid="{7F739DF3-AE70-5648-ABAC-6400F7C2E419}"/>
   </bookViews>
   <sheets>
     <sheet name="UWE_Constructions" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="98">
   <si>
     <t>Element</t>
   </si>
@@ -200,9 +200,6 @@
   </si>
   <si>
     <t>GB.ENG.MFH.01.Gen.ReEx.001.001</t>
-  </si>
-  <si>
-    <t>Pitched with Gables</t>
   </si>
   <si>
     <t>GB.ENG.MFH.02.Gen.ReEx.001.001</t>
@@ -1276,13 +1273,13 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>49</v>
@@ -1296,13 +1293,13 @@
         <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>49</v>
@@ -1316,13 +1313,13 @@
         <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>49</v>
@@ -1335,14 +1332,14 @@
       <c r="A5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>54</v>
+      <c r="B5" t="s">
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>49</v>
@@ -1353,16 +1350,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="2" t="s">
         <v>54</v>
       </c>
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>49</v>
@@ -1373,16 +1370,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>49</v>
@@ -1393,16 +1390,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>49</v>
@@ -1413,16 +1410,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>49</v>
@@ -1433,16 +1430,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>49</v>
@@ -1453,16 +1450,16 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>49</v>
@@ -1473,16 +1470,16 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>49</v>
@@ -1493,16 +1490,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>49</v>
@@ -1513,16 +1510,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>49</v>
@@ -1533,16 +1530,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>49</v>
@@ -1553,16 +1550,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>49</v>
@@ -1573,16 +1570,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>49</v>
@@ -1593,16 +1590,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>49</v>
@@ -1613,16 +1610,16 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>49</v>
@@ -1633,16 +1630,16 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>49</v>
@@ -1653,16 +1650,16 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>49</v>
@@ -1673,16 +1670,16 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>49</v>
@@ -1693,16 +1690,16 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>49</v>
@@ -1713,16 +1710,16 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>49</v>
@@ -1733,16 +1730,16 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>49</v>
@@ -1753,16 +1750,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>49</v>
@@ -1773,16 +1770,16 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B27" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>49</v>
@@ -1793,16 +1790,16 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>49</v>
@@ -1829,10 +1826,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>98</v>
       </c>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
@@ -1840,7 +1837,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -1848,7 +1845,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -1856,7 +1853,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -1864,7 +1861,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -1873,7 +1870,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1882,7 +1879,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
@@ -1891,7 +1888,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B8" t="s">
         <v>25</v>
@@ -1899,7 +1896,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
@@ -1907,7 +1904,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
@@ -1915,7 +1912,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B11" t="s">
         <v>29</v>
@@ -1923,7 +1920,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
@@ -1931,7 +1928,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -1939,7 +1936,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
         <v>36</v>
@@ -1947,7 +1944,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B15" t="s">
         <v>37</v>
@@ -1955,7 +1952,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
         <v>39</v>
@@ -1963,7 +1960,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B17" t="s">
         <v>40</v>
@@ -1971,7 +1968,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
         <v>40</v>
@@ -1979,7 +1976,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B19" t="s">
         <v>41</v>
@@ -1987,7 +1984,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
         <v>41</v>

</xml_diff>